<commit_message>
Add optional key_type coercion for mapped key fields
</commit_message>
<xml_diff>
--- a/mappings/workday_mapping_sample.xlsx
+++ b/mappings/workday_mapping_sample.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="table_map" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="field_map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="value_map" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,6 +525,11 @@
           <t>compare</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>key_type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -552,6 +558,11 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -664,6 +675,11 @@
       <c r="F6" t="b">
         <v>1</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -748,6 +764,11 @@
       <c r="F9" t="b">
         <v>1</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -803,6 +824,130 @@
       </c>
       <c r="F11" t="b">
         <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>table_value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>canonical_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>wd_dev.worker_core</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>active_flag</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>wd_dev.worker_core</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>active_flag</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>wd_prod.worker_core</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>wd_prod.worker_core</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>